<commit_message>
WS-7: testes do modelo padrão e da criação do zero; colunas calculadas declaradas na tabela; colunas ocultas não recebem dados
</commit_message>
<xml_diff>
--- a/src/modelos/xlsx_b/modelo_padrao.xlsx
+++ b/src/modelos/xlsx_b/modelo_padrao.xlsx
@@ -857,9 +857,13 @@
     <tableColumn id="20" name="Depósitos Recursais"/>
     <tableColumn id="21" name="Garantias Processuais"/>
     <tableColumn id="22" name="Resultado"/>
-    <tableColumn id="23" name="Valor Economizado"/>
+    <tableColumn id="23" name="Valor Economizado">
+      <calculatedColumnFormula>IF(OR(tblProcessos[[#This Row],[Ativo]]&lt;&gt;"Não",tblProcessos[[#This Row],[Valor da Causa]]="",tblProcessos[[#This Row],[Valor Estimado]]=""),"",tblProcessos[[#This Row],[Valor da Causa]]-tblProcessos[[#This Row],[Valor Estimado]])</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="24" name="Data do trânsito em julgado"/>
-    <tableColumn id="25" name="Taxa de resolução (em dias)"/>
+    <tableColumn id="25" name="Taxa de resolução (em dias)">
+      <calculatedColumnFormula>IF(OR(tblProcessos[[#This Row],[Data do trânsito em julgado]]="",tblProcessos[[#This Row],[Data do Ajuizamento]]=""),"",tblProcessos[[#This Row],[Data do trânsito em julgado]]-tblProcessos[[#This Row],[Data do Ajuizamento]])</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="26" name="Houve recurso da empresa?"/>
     <tableColumn id="27" name="Percentual de êxito"/>
     <tableColumn id="28" name="Reclamante terceirizado?"/>
@@ -1576,12 +1580,9 @@
           <t>Fator de correção</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Multiplica o valor da causa total (1 = sem correção).</t>
+          <t>Multiplica o valor da causa total (vazio = sem correção).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WS-7: aviso agregado andamento_ja_presente, modelo com textos compartilhados, avisos de coluna Andamentos ausente e filtro ativo
</commit_message>
<xml_diff>
--- a/src/modelos/xlsx_b/modelo_padrao.xlsx
+++ b/src/modelos/xlsx_b/modelo_padrao.xlsx
@@ -17,6 +17,431 @@
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="140">
+  <si>
+    <t>Número do Processo</t>
+  </si>
+  <si>
+    <t>Autor(es)</t>
+  </si>
+  <si>
+    <t>Réu(s)</t>
+  </si>
+  <si>
+    <t>Vara</t>
+  </si>
+  <si>
+    <t>Município</t>
+  </si>
+  <si>
+    <t>Tribunal</t>
+  </si>
+  <si>
+    <t>Data do Ajuizamento</t>
+  </si>
+  <si>
+    <t>Área do Direito</t>
+  </si>
+  <si>
+    <t>Matéria Principal</t>
+  </si>
+  <si>
+    <t>Objeto</t>
+  </si>
+  <si>
+    <t>Valor da Causa</t>
+  </si>
+  <si>
+    <t>Andamentos</t>
+  </si>
+  <si>
+    <t>Situação</t>
+  </si>
+  <si>
+    <t>Ativo</t>
+  </si>
+  <si>
+    <t>Valor Arbitrado em Juízo</t>
+  </si>
+  <si>
+    <t>Probabilidade</t>
+  </si>
+  <si>
+    <t>Valor Estimado</t>
+  </si>
+  <si>
+    <t>Valor da Execução</t>
+  </si>
+  <si>
+    <t>Custas Processuais</t>
+  </si>
+  <si>
+    <t>Depósitos Recursais</t>
+  </si>
+  <si>
+    <t>Garantias Processuais</t>
+  </si>
+  <si>
+    <t>Resultado</t>
+  </si>
+  <si>
+    <t>Valor Economizado</t>
+  </si>
+  <si>
+    <t>Data do trânsito em julgado</t>
+  </si>
+  <si>
+    <t>Taxa de resolução (em dias)</t>
+  </si>
+  <si>
+    <t>Houve recurso da empresa?</t>
+  </si>
+  <si>
+    <t>Percentual de êxito</t>
+  </si>
+  <si>
+    <t>Reclamante terceirizado?</t>
+  </si>
+  <si>
+    <t>Outra(s) Parte(s)</t>
+  </si>
+  <si>
+    <t>Momento Atual</t>
+  </si>
+  <si>
+    <t>Último Andamento</t>
+  </si>
+  <si>
+    <t>Data de Citação</t>
+  </si>
+  <si>
+    <t>Fase</t>
+  </si>
+  <si>
+    <t>Classe</t>
+  </si>
+  <si>
+    <t>Assunto</t>
+  </si>
+  <si>
+    <t>Valor do Acordo</t>
+  </si>
+  <si>
+    <t>Observações</t>
+  </si>
+  <si>
+    <t>Parâmetro</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>Número de funcionários (headcount)</t>
+  </si>
+  <si>
+    <t>Usado em 'Litígios por 100 funcionários'.</t>
+  </si>
+  <si>
+    <t>Data de referência</t>
+  </si>
+  <si>
+    <t>Data-base do relatório; usada nos 'novos ajuizamentos em 12 meses'.</t>
+  </si>
+  <si>
+    <t>Fator de correção</t>
+  </si>
+  <si>
+    <t>Multiplica o valor da causa total (vazio = sem correção).</t>
+  </si>
+  <si>
+    <t>Empresas do grupo</t>
+  </si>
+  <si>
+    <t>Nomes separados por ponto e vírgula.</t>
+  </si>
+  <si>
+    <t>Indicador</t>
+  </si>
+  <si>
+    <t>Como é calculado</t>
+  </si>
+  <si>
+    <t>Acervo</t>
+  </si>
+  <si>
+    <t>Total de processos</t>
+  </si>
+  <si>
+    <t>Linhas com número de processo.</t>
+  </si>
+  <si>
+    <t>Processos ativos</t>
+  </si>
+  <si>
+    <t>Coluna Ativo = Sim.</t>
+  </si>
+  <si>
+    <t>Processos encerrados</t>
+  </si>
+  <si>
+    <t>Coluna Ativo = Não.</t>
+  </si>
+  <si>
+    <t>Litígios por 100 funcionários</t>
+  </si>
+  <si>
+    <t>Total de processos ÷ número de funcionários × 100 (precisa do headcount em Parâmetros).</t>
+  </si>
+  <si>
+    <t>Novos ajuizamentos em 12 meses</t>
+  </si>
+  <si>
+    <t>Ajuizados nos 12 meses até a data de referência (Parâmetros).</t>
+  </si>
+  <si>
+    <t>Tempo e recursos</t>
+  </si>
+  <si>
+    <t>Tempo médio de resolução (dias)</t>
+  </si>
+  <si>
+    <t>Média da Taxa de resolução (trânsito em julgado − ajuizamento).</t>
+  </si>
+  <si>
+    <t>Mediana do tempo de resolução (dias)</t>
+  </si>
+  <si>
+    <t>Mediana da Taxa de resolução.</t>
+  </si>
+  <si>
+    <t>Processos com recurso da empresa</t>
+  </si>
+  <si>
+    <t>Coluna Houve recurso da empresa? = Sim.</t>
+  </si>
+  <si>
+    <t>Processos decididos</t>
+  </si>
+  <si>
+    <t>Soma dos cinco desfechos abaixo (não conta extinção sem mérito nem incompetência).</t>
+  </si>
+  <si>
+    <t>Taxa de recurso</t>
+  </si>
+  <si>
+    <t>Processos com recurso da empresa ÷ decididos.</t>
+  </si>
+  <si>
+    <t>Resultados</t>
+  </si>
+  <si>
+    <t>Improcedentes</t>
+  </si>
+  <si>
+    <t>Coluna Resultado = Improcedente.</t>
+  </si>
+  <si>
+    <t>Arquivadas / desistência</t>
+  </si>
+  <si>
+    <t>Coluna Resultado = Arquivado / desistência.</t>
+  </si>
+  <si>
+    <t>Acordos</t>
+  </si>
+  <si>
+    <t>Coluna Resultado = Acordo.</t>
+  </si>
+  <si>
+    <t>Parcialmente procedentes</t>
+  </si>
+  <si>
+    <t>Coluna Resultado = Parcialmente procedente.</t>
+  </si>
+  <si>
+    <t>Procedentes</t>
+  </si>
+  <si>
+    <t>Coluna Resultado = Procedente.</t>
+  </si>
+  <si>
+    <t>Taxa de êxito</t>
+  </si>
+  <si>
+    <t>(Improcedentes + arquivadas) ÷ decididos.</t>
+  </si>
+  <si>
+    <t>% por acordo</t>
+  </si>
+  <si>
+    <t>Acordos ÷ decididos.</t>
+  </si>
+  <si>
+    <t>Financeiro</t>
+  </si>
+  <si>
+    <t>Valor da causa total</t>
+  </si>
+  <si>
+    <t>Soma da coluna Valor da Causa.</t>
+  </si>
+  <si>
+    <t>Valor da causa total corrigido</t>
+  </si>
+  <si>
+    <t>Valor da causa × fator de correção (Parâmetros).</t>
+  </si>
+  <si>
+    <t>Valor da causa dos encerrados</t>
+  </si>
+  <si>
+    <t>Processos com Ativo = Não.</t>
+  </si>
+  <si>
+    <t>Encerrados com valor realizado lançado</t>
+  </si>
+  <si>
+    <t>Têm valor arbitrado ou, se este estiver vazio, valor da execução.</t>
+  </si>
+  <si>
+    <t>Encerrados sem valor lançado (fora da economia)</t>
+  </si>
+  <si>
+    <t>Ficam fora da economia para não inflá-la (acordo sem valor lançado etc.).</t>
+  </si>
+  <si>
+    <t>Valor da causa dos encerrados com valor lançado</t>
+  </si>
+  <si>
+    <t>Base da economia efetiva.</t>
+  </si>
+  <si>
+    <t>Valor realizado dos encerrados</t>
+  </si>
+  <si>
+    <t>Valor arbitrado em juízo, ou o valor da execução quando o arbitrado está vazio.</t>
+  </si>
+  <si>
+    <t>Economia efetiva</t>
+  </si>
+  <si>
+    <t>Valor da causa − valor realizado, só dos encerrados com valor lançado.</t>
+  </si>
+  <si>
+    <t>Processos por situação</t>
+  </si>
+  <si>
+    <t>Processos</t>
+  </si>
+  <si>
+    <t>Encerrado</t>
+  </si>
+  <si>
+    <t>Suspenso</t>
+  </si>
+  <si>
+    <t>Processos por resultado</t>
+  </si>
+  <si>
+    <t>Procedente</t>
+  </si>
+  <si>
+    <t>Parcialmente procedente</t>
+  </si>
+  <si>
+    <t>Improcedente</t>
+  </si>
+  <si>
+    <t>Acordo</t>
+  </si>
+  <si>
+    <t>Extinto sem resolução de mérito</t>
+  </si>
+  <si>
+    <t>Arquivado / desistência</t>
+  </si>
+  <si>
+    <t>Incompetência declarada</t>
+  </si>
+  <si>
+    <t>Processos por área</t>
+  </si>
+  <si>
+    <t>Trabalhista</t>
+  </si>
+  <si>
+    <t>Cível</t>
+  </si>
+  <si>
+    <t>Consumidor</t>
+  </si>
+  <si>
+    <t>Tributário</t>
+  </si>
+  <si>
+    <t>Administrativo</t>
+  </si>
+  <si>
+    <t>Ambiental</t>
+  </si>
+  <si>
+    <t>Empresarial</t>
+  </si>
+  <si>
+    <t>Imobiliário</t>
+  </si>
+  <si>
+    <t>Contratual</t>
+  </si>
+  <si>
+    <t>Processual</t>
+  </si>
+  <si>
+    <t>Previdenciário</t>
+  </si>
+  <si>
+    <t>Processos por probabilidade</t>
+  </si>
+  <si>
+    <t>Possível</t>
+  </si>
+  <si>
+    <t>Provável</t>
+  </si>
+  <si>
+    <t>Remota</t>
+  </si>
+  <si>
+    <t>Resumo da carteira</t>
+  </si>
+  <si>
+    <t>Ativos</t>
+  </si>
+  <si>
+    <t>Data-base</t>
+  </si>
+  <si>
+    <t>Encerrados</t>
+  </si>
+  <si>
+    <t>Valor da causa</t>
+  </si>
+  <si>
+    <t>Valor estimado</t>
+  </si>
+  <si>
+    <t>Valor economizado</t>
+  </si>
+  <si>
+    <t>Coluna de origem</t>
+  </si>
+  <si>
+    <t>Processo</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1241,190 +1666,116 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Número do Processo</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Autor(es)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Réu(s)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Vara</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Município</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Tribunal</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Data do Ajuizamento</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Área do Direito</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Matéria Principal</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Objeto</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Valor da Causa</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Andamentos</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Situação</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Valor Arbitrado em Juízo</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Probabilidade</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Valor Estimado</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Valor da Execução</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Custas Processuais</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Depósitos Recursais</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Garantias Processuais</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Resultado</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Valor Economizado</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Data do trânsito em julgado</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Taxa de resolução (em dias)</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Houve recurso da empresa?</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>Percentual de êxito</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Reclamante terceirizado?</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Outra(s) Parte(s)</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Momento Atual</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Último Andamento</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>Data de Citação</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Fase</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>Classe</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>Assunto</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>Valor do Acordo</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>Observações</t>
-        </is>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="2">
@@ -1538,64 +1889,44 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>Parâmetro</t>
-        </is>
-      </c>
-      <c r="B1" s="8" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
+      <c r="A1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Número de funcionários (headcount)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Usado em 'Litígios por 100 funcionários'.</t>
-        </is>
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Data de referência</t>
-        </is>
+      <c r="A3" t="s">
+        <v>41</v>
       </c>
       <c r="B3" s="9" t="n"/>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Data-base do relatório; usada nos 'novos ajuizamentos em 12 meses'.</t>
-        </is>
+      <c r="C3" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Fator de correção</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Multiplica o valor da causa total (vazio = sem correção).</t>
-        </is>
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Empresas do grupo</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Nomes separados por ponto e vírgula.</t>
-        </is>
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1618,467 +1949,347 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>Indicador</t>
-        </is>
-      </c>
-      <c r="B1" s="8" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="C1" s="8" t="inlineStr">
-        <is>
-          <t>Como é calculado</t>
-        </is>
+      <c r="A1" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>Acervo</t>
-        </is>
+      <c r="A2" s="10" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Total de processos</t>
-        </is>
+      <c r="A3" t="s">
+        <v>50</v>
       </c>
       <c r="B3" s="11">
         <f>COUNTA(tblProcessos[Número do Processo])</f>
         <v/>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Linhas com número de processo.</t>
-        </is>
+      <c r="C3" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Processos ativos</t>
-        </is>
+      <c r="A4" t="s">
+        <v>52</v>
       </c>
       <c r="B4" s="11">
         <f>COUNTIFS(tblProcessos[Ativo],"Sim")</f>
         <v/>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Coluna Ativo = Sim.</t>
-        </is>
+      <c r="C4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Processos encerrados</t>
-        </is>
+      <c r="A5" t="s">
+        <v>54</v>
       </c>
       <c r="B5" s="11">
         <f>COUNTIFS(tblProcessos[Ativo],"Não")</f>
         <v/>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Coluna Ativo = Não.</t>
-        </is>
+      <c r="C5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Litígios por 100 funcionários</t>
-        </is>
+      <c r="A6" t="s">
+        <v>56</v>
       </c>
       <c r="B6" s="12">
         <f>IF(N('Parâmetros'!$B$2)&gt;0,B3/'Parâmetros'!$B$2*100,"")</f>
         <v/>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Total de processos ÷ número de funcionários × 100 (precisa do headcount em Parâmetros).</t>
-        </is>
+      <c r="C6" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Novos ajuizamentos em 12 meses</t>
-        </is>
+      <c r="A7" t="s">
+        <v>58</v>
       </c>
       <c r="B7" s="11">
         <f>IF(N('Parâmetros'!$B$3)&gt;0,COUNTIFS(tblProcessos[Data do Ajuizamento],"&gt;"&amp;EDATE('Parâmetros'!$B$3,-12),tblProcessos[Data do Ajuizamento],"&lt;="&amp;'Parâmetros'!$B$3),"")</f>
         <v/>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Ajuizados nos 12 meses até a data de referência (Parâmetros).</t>
-        </is>
+      <c r="C7" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Tempo e recursos</t>
-        </is>
+      <c r="A9" s="10" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Tempo médio de resolução (dias)</t>
-        </is>
+      <c r="A10" t="s">
+        <v>61</v>
       </c>
       <c r="B10" s="12">
         <f>IFERROR(AVERAGE(tblProcessos[[Taxa de resolução (em dias)]]),"")</f>
         <v/>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Média da Taxa de resolução (trânsito em julgado − ajuizamento).</t>
-        </is>
+      <c r="C10" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Mediana do tempo de resolução (dias)</t>
-        </is>
+      <c r="A11" t="s">
+        <v>63</v>
       </c>
       <c r="B11" s="12">
         <f>IFERROR(MEDIAN(tblProcessos[[Taxa de resolução (em dias)]]),"")</f>
         <v/>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Mediana da Taxa de resolução.</t>
-        </is>
+      <c r="C11" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Processos com recurso da empresa</t>
-        </is>
+      <c r="A12" t="s">
+        <v>65</v>
       </c>
       <c r="B12" s="11">
         <f>COUNTIFS(tblProcessos[[Houve recurso da empresa?]],"Sim")</f>
         <v/>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Coluna Houve recurso da empresa? = Sim.</t>
-        </is>
+      <c r="C12" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Processos decididos</t>
-        </is>
+      <c r="A13" t="s">
+        <v>67</v>
       </c>
       <c r="B13" s="11">
         <f>B17+B18+B19+B20+B21</f>
         <v/>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Soma dos cinco desfechos abaixo (não conta extinção sem mérito nem incompetência).</t>
-        </is>
+      <c r="C13" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Taxa de recurso</t>
-        </is>
+      <c r="A14" t="s">
+        <v>69</v>
       </c>
       <c r="B14" s="13">
         <f>IF(B13&gt;0,B12/B13,"")</f>
         <v/>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Processos com recurso da empresa ÷ decididos.</t>
-        </is>
+      <c r="C14" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>Resultados</t>
-        </is>
+      <c r="A16" s="10" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Improcedentes</t>
-        </is>
+      <c r="A17" t="s">
+        <v>72</v>
       </c>
       <c r="B17" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],"Improcedente")</f>
         <v/>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Coluna Resultado = Improcedente.</t>
-        </is>
+      <c r="C17" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Arquivadas / desistência</t>
-        </is>
+      <c r="A18" t="s">
+        <v>74</v>
       </c>
       <c r="B18" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],"Arquivado / desistência")</f>
         <v/>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Coluna Resultado = Arquivado / desistência.</t>
-        </is>
+      <c r="C18" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Acordos</t>
-        </is>
+      <c r="A19" t="s">
+        <v>76</v>
       </c>
       <c r="B19" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],"Acordo")</f>
         <v/>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Coluna Resultado = Acordo.</t>
-        </is>
+      <c r="C19" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Parcialmente procedentes</t>
-        </is>
+      <c r="A20" t="s">
+        <v>78</v>
       </c>
       <c r="B20" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],"Parcialmente procedente")</f>
         <v/>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Coluna Resultado = Parcialmente procedente.</t>
-        </is>
+      <c r="C20" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Procedentes</t>
-        </is>
+      <c r="A21" t="s">
+        <v>80</v>
       </c>
       <c r="B21" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],"Procedente")</f>
         <v/>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Coluna Resultado = Procedente.</t>
-        </is>
+      <c r="C21" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Taxa de êxito</t>
-        </is>
+      <c r="A22" t="s">
+        <v>82</v>
       </c>
       <c r="B22" s="13">
         <f>IF(B13&gt;0,(B17+B18)/B13,"")</f>
         <v/>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>(Improcedentes + arquivadas) ÷ decididos.</t>
-        </is>
+      <c r="C22" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>% por acordo</t>
-        </is>
+      <c r="A23" t="s">
+        <v>84</v>
       </c>
       <c r="B23" s="13">
         <f>IF(B13&gt;0,B19/B13,"")</f>
         <v/>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Acordos ÷ decididos.</t>
-        </is>
+      <c r="C23" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Financeiro</t>
-        </is>
+      <c r="A25" s="10" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Valor da causa total</t>
-        </is>
+      <c r="A26" t="s">
+        <v>87</v>
       </c>
       <c r="B26" s="14">
         <f>SUM(tblProcessos[Valor da Causa])</f>
         <v/>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Soma da coluna Valor da Causa.</t>
-        </is>
+      <c r="C26" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Valor da causa total corrigido</t>
-        </is>
+      <c r="A27" t="s">
+        <v>89</v>
       </c>
       <c r="B27" s="14">
         <f>IF(N('Parâmetros'!$B$4)&gt;0,B26*'Parâmetros'!$B$4,B26)</f>
         <v/>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Valor da causa × fator de correção (Parâmetros).</t>
-        </is>
+      <c r="C27" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Valor da causa dos encerrados</t>
-        </is>
+      <c r="A28" t="s">
+        <v>91</v>
       </c>
       <c r="B28" s="14">
         <f>SUMIFS(tblProcessos[Valor da Causa],tblProcessos[Ativo],"Não")</f>
         <v/>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Processos com Ativo = Não.</t>
-        </is>
+      <c r="C28" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Encerrados com valor realizado lançado</t>
-        </is>
+      <c r="A29" t="s">
+        <v>93</v>
       </c>
       <c r="B29" s="11">
         <f>COUNTIFS(tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"&lt;&gt;")+COUNTIFS(tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"",tblProcessos[Valor da Execução],"&lt;&gt;")</f>
         <v/>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Têm valor arbitrado ou, se este estiver vazio, valor da execução.</t>
-        </is>
+      <c r="C29" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Encerrados sem valor lançado (fora da economia)</t>
-        </is>
+      <c r="A30" t="s">
+        <v>95</v>
       </c>
       <c r="B30" s="11">
         <f>B5-B29</f>
         <v/>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Ficam fora da economia para não inflá-la (acordo sem valor lançado etc.).</t>
-        </is>
+      <c r="C30" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Valor da causa dos encerrados com valor lançado</t>
-        </is>
+      <c r="A31" t="s">
+        <v>97</v>
       </c>
       <c r="B31" s="14">
         <f>SUMIFS(tblProcessos[Valor da Causa],tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"&lt;&gt;")+SUMIFS(tblProcessos[Valor da Causa],tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"",tblProcessos[Valor da Execução],"&lt;&gt;")</f>
         <v/>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Base da economia efetiva.</t>
-        </is>
+      <c r="C31" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Valor realizado dos encerrados</t>
-        </is>
+      <c r="A32" t="s">
+        <v>99</v>
       </c>
       <c r="B32" s="14">
         <f>SUMIFS(tblProcessos[Valor Arbitrado em Juízo],tblProcessos[Ativo],"Não")+SUMIFS(tblProcessos[Valor da Execução],tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"")</f>
         <v/>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Valor arbitrado em juízo, ou o valor da execução quando o arbitrado está vazio.</t>
-        </is>
+      <c r="C32" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Economia efetiva</t>
-        </is>
+      <c r="A33" t="s">
+        <v>101</v>
       </c>
       <c r="B33" s="14">
         <f>B31-B32</f>
         <v/>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Valor da causa − valor realizado, só dos encerrados com valor lançado.</t>
-        </is>
+      <c r="C33" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Processos por situação</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Processos</t>
-        </is>
+      <c r="A35" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
+      <c r="A36" t="s">
+        <v>13</v>
       </c>
       <c r="B36" s="11">
         <f>COUNTIFS(tblProcessos[Situação],A36)</f>
@@ -2086,10 +2297,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Encerrado</t>
-        </is>
+      <c r="A37" t="s">
+        <v>105</v>
       </c>
       <c r="B37" s="11">
         <f>COUNTIFS(tblProcessos[Situação],A37)</f>
@@ -2097,10 +2306,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Suspenso</t>
-        </is>
+      <c r="A38" t="s">
+        <v>106</v>
       </c>
       <c r="B38" s="11">
         <f>COUNTIFS(tblProcessos[Situação],A38)</f>
@@ -2108,22 +2315,16 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>Processos por resultado</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>Processos</t>
-        </is>
+      <c r="A40" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Procedente</t>
-        </is>
+      <c r="A41" t="s">
+        <v>108</v>
       </c>
       <c r="B41" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],A41)</f>
@@ -2131,10 +2332,8 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Parcialmente procedente</t>
-        </is>
+      <c r="A42" t="s">
+        <v>109</v>
       </c>
       <c r="B42" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],A42)</f>
@@ -2142,10 +2341,8 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Improcedente</t>
-        </is>
+      <c r="A43" t="s">
+        <v>110</v>
       </c>
       <c r="B43" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],A43)</f>
@@ -2153,10 +2350,8 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Acordo</t>
-        </is>
+      <c r="A44" t="s">
+        <v>111</v>
       </c>
       <c r="B44" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],A44)</f>
@@ -2164,10 +2359,8 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Extinto sem resolução de mérito</t>
-        </is>
+      <c r="A45" t="s">
+        <v>112</v>
       </c>
       <c r="B45" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],A45)</f>
@@ -2175,10 +2368,8 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Arquivado / desistência</t>
-        </is>
+      <c r="A46" t="s">
+        <v>113</v>
       </c>
       <c r="B46" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],A46)</f>
@@ -2186,10 +2377,8 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Incompetência declarada</t>
-        </is>
+      <c r="A47" t="s">
+        <v>114</v>
       </c>
       <c r="B47" s="11">
         <f>COUNTIFS(tblProcessos[Resultado],A47)</f>
@@ -2197,22 +2386,16 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>Processos por área</t>
-        </is>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>Processos</t>
-        </is>
+      <c r="A49" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Trabalhista</t>
-        </is>
+      <c r="A50" t="s">
+        <v>116</v>
       </c>
       <c r="B50" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A50)</f>
@@ -2220,10 +2403,8 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Cível</t>
-        </is>
+      <c r="A51" t="s">
+        <v>117</v>
       </c>
       <c r="B51" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A51)</f>
@@ -2231,10 +2412,8 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Consumidor</t>
-        </is>
+      <c r="A52" t="s">
+        <v>118</v>
       </c>
       <c r="B52" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A52)</f>
@@ -2242,10 +2421,8 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Tributário</t>
-        </is>
+      <c r="A53" t="s">
+        <v>119</v>
       </c>
       <c r="B53" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A53)</f>
@@ -2253,10 +2430,8 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Administrativo</t>
-        </is>
+      <c r="A54" t="s">
+        <v>120</v>
       </c>
       <c r="B54" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A54)</f>
@@ -2264,10 +2439,8 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Ambiental</t>
-        </is>
+      <c r="A55" t="s">
+        <v>121</v>
       </c>
       <c r="B55" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A55)</f>
@@ -2275,10 +2448,8 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Empresarial</t>
-        </is>
+      <c r="A56" t="s">
+        <v>122</v>
       </c>
       <c r="B56" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A56)</f>
@@ -2286,10 +2457,8 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Imobiliário</t>
-        </is>
+      <c r="A57" t="s">
+        <v>123</v>
       </c>
       <c r="B57" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A57)</f>
@@ -2297,10 +2466,8 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Contratual</t>
-        </is>
+      <c r="A58" t="s">
+        <v>124</v>
       </c>
       <c r="B58" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A58)</f>
@@ -2308,10 +2475,8 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Processual</t>
-        </is>
+      <c r="A59" t="s">
+        <v>125</v>
       </c>
       <c r="B59" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A59)</f>
@@ -2319,10 +2484,8 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Previdenciário</t>
-        </is>
+      <c r="A60" t="s">
+        <v>126</v>
       </c>
       <c r="B60" s="11">
         <f>COUNTIFS(tblProcessos[Área do Direito],A60)</f>
@@ -2330,22 +2493,16 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="inlineStr">
-        <is>
-          <t>Processos por probabilidade</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>Processos</t>
-        </is>
+      <c r="A62" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Possível</t>
-        </is>
+      <c r="A63" t="s">
+        <v>128</v>
       </c>
       <c r="B63" s="11">
         <f>COUNTIFS(tblProcessos[Probabilidade],A63)</f>
@@ -2353,10 +2510,8 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Provável</t>
-        </is>
+      <c r="A64" t="s">
+        <v>129</v>
       </c>
       <c r="B64" s="11">
         <f>COUNTIFS(tblProcessos[Probabilidade],A64)</f>
@@ -2364,10 +2519,8 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Remota</t>
-        </is>
+      <c r="A65" t="s">
+        <v>130</v>
       </c>
       <c r="B65" s="11">
         <f>COUNTIFS(tblProcessos[Probabilidade],A65)</f>
@@ -2399,32 +2552,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Resumo da carteira</t>
-        </is>
+      <c r="A1" s="15" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>Processos</t>
-        </is>
-      </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>Ativos</t>
-        </is>
-      </c>
-      <c r="E3" s="16" t="inlineStr">
-        <is>
-          <t>Taxa de êxito</t>
-        </is>
-      </c>
-      <c r="G3" s="16" t="inlineStr">
-        <is>
-          <t>Economia efetiva</t>
-        </is>
+      <c r="A3" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="4">
@@ -2470,40 +2613,26 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>Data-base</t>
-        </is>
-      </c>
-      <c r="B1" s="20" t="inlineStr">
-        <is>
-          <t>Processos</t>
-        </is>
-      </c>
-      <c r="C1" s="20" t="inlineStr">
-        <is>
-          <t>Ativos</t>
-        </is>
-      </c>
-      <c r="D1" s="20" t="inlineStr">
-        <is>
-          <t>Encerrados</t>
-        </is>
-      </c>
-      <c r="E1" s="20" t="inlineStr">
-        <is>
-          <t>Valor da causa</t>
-        </is>
-      </c>
-      <c r="F1" s="20" t="inlineStr">
-        <is>
-          <t>Valor estimado</t>
-        </is>
-      </c>
-      <c r="G1" s="20" t="inlineStr">
-        <is>
-          <t>Valor economizado</t>
-        </is>
+      <c r="A1" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="F1" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="G1" s="20" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="2">
@@ -2538,20 +2667,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>Coluna de origem</t>
-        </is>
-      </c>
-      <c r="B1" s="20" t="inlineStr">
-        <is>
-          <t>Processo</t>
-        </is>
-      </c>
-      <c r="C1" s="20" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
+      <c r="A1" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
WS-7: cabeçalhos do Histórico como o dashboard lê, retrato do ciclo via historico.retrato, gerador de exemplos, conferência manual e RFC
</commit_message>
<xml_diff>
--- a/src/modelos/xlsx_b/modelo_padrao.xlsx
+++ b/src/modelos/xlsx_b/modelo_padrao.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="140">
   <si>
     <t>Número do Processo</t>
   </si>
@@ -403,6 +403,9 @@
     <t>Previdenciário</t>
   </si>
   <si>
+    <t>Família e Sucessões</t>
+  </si>
+  <si>
     <t>Processos por probabilidade</t>
   </si>
   <si>
@@ -422,9 +425,6 @@
   </si>
   <si>
     <t>Data-base</t>
-  </si>
-  <si>
-    <t>Encerrados</t>
   </si>
   <si>
     <t>Valor da causa</t>
@@ -868,12 +868,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Indicadores'!$A$50:$A$60</f>
+              <f>'Indicadores'!$A$50:$A$61</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Indicadores'!$B$50:$B$60</f>
+              <f>'Indicadores'!$B$50:$B$61</f>
             </numRef>
           </val>
         </ser>
@@ -959,12 +959,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Indicadores'!$A$63:$A$65</f>
+              <f>'Indicadores'!$A$64:$A$66</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Indicadores'!$B$63:$B$65</f>
+              <f>'Indicadores'!$B$64:$B$66</f>
             </numRef>
           </val>
         </ser>
@@ -1311,9 +1311,9 @@
   <autoFilter ref="A1:G2"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Data-base"/>
-    <tableColumn id="2" name="Processos"/>
-    <tableColumn id="3" name="Ativos"/>
-    <tableColumn id="4" name="Encerrados"/>
+    <tableColumn id="2" name="Total de processos"/>
+    <tableColumn id="3" name="Processos ativos"/>
+    <tableColumn id="4" name="Processos encerrados"/>
     <tableColumn id="5" name="Valor da causa"/>
     <tableColumn id="6" name="Valor estimado"/>
     <tableColumn id="7" name="Valor economizado"/>
@@ -1851,7 +1851,7 @@
       <formula1>"Procedente,Parcialmente procedente,Improcedente,Acordo,Extinto sem resolução de mérito,Arquivado / desistência,Incompetência declarada"</formula1>
     </dataValidation>
     <dataValidation sqref="H2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Área do Direito" error="Valor fora da lista padrão. Manter assim?" type="list" errorStyle="warning">
-      <formula1>"Trabalhista,Cível,Consumidor,Tributário,Administrativo,Ambiental,Empresarial,Imobiliário,Contratual,Processual,Previdenciário"</formula1>
+      <formula1>"Trabalhista,Cível,Consumidor,Tributário,Administrativo,Ambiental,Empresarial,Imobiliário,Contratual,Processual,Previdenciário,Família e Sucessões"</formula1>
     </dataValidation>
     <dataValidation sqref="N2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ativo" error="Valor fora da lista padrão. Manter assim?" type="list" errorStyle="warning">
       <formula1>"Sim,Não"</formula1>
@@ -1940,7 +1940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2492,21 +2492,21 @@
         <v/>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="10" t="s">
+    <row r="61">
+      <c r="A61" t="s">
         <v>127</v>
       </c>
-      <c r="B62" s="8" t="s">
+      <c r="B61" s="11">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A61)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="B63" s="8" t="s">
         <v>104</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="s">
-        <v>128</v>
-      </c>
-      <c r="B63" s="11">
-        <f>COUNTIFS(tblProcessos[Probabilidade],A63)</f>
-        <v/>
       </c>
     </row>
     <row r="64">
@@ -2524,6 +2524,15 @@
       </c>
       <c r="B65" s="11">
         <f>COUNTIFS(tblProcessos[Probabilidade],A65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>131</v>
+      </c>
+      <c r="B66" s="11">
+        <f>COUNTIFS(tblProcessos[Probabilidade],A66)</f>
         <v/>
       </c>
     </row>
@@ -2553,7 +2562,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3">
@@ -2561,7 +2570,7 @@
         <v>104</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E3" s="16" t="s">
         <v>82</v>
@@ -2614,16 +2623,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>104</v>
+        <v>50</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>132</v>
+        <v>52</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>134</v>
+        <v>54</v>
       </c>
       <c r="E1" s="20" t="s">
         <v>135</v>

</xml_diff>

<commit_message>
Migração de planilhas de contingências: campos de contingência no modelo B, leitor, relatório de lacunas e painel
- ficha: grupo contingencia (passivo potencial e atualizado, ativo potencial, % e valor da provisão, depósito judicial, CNPJ, pagamento, justificativa) e derivação depósito/percentual
- leitor: sinônimos, valores (R$, %, sim/não, grau + justificativa), fórmulas simples calculadas, rodapé/legenda fora, Natureza da ação como assunto
- lacunas.py e quadro 'O que falta para a transição' nas telas de migração e conferência; aba 'Faltas da migração' na planilha
- modelo B: colunas 38 a 46, indicadores e gráfico de contingência; painel HTML com bloco de contingência
- testes com planilha fictícia (tests/test_contingencias.py); '(não usar)' na migração passa a excluir a coluna de fato

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/modelos/xlsx_b/modelo_padrao.xlsx
+++ b/src/modelos/xlsx_b/modelo_padrao.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Histórico" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campos não migrados" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faltas da migração" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campos não migrados" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="184">
   <si>
     <t>Número do Processo</t>
   </si>
@@ -133,6 +134,33 @@
     <t>Observações</t>
   </si>
   <si>
+    <t>Passivo Potencial</t>
+  </si>
+  <si>
+    <t>Passivo Potencial Atualizado</t>
+  </si>
+  <si>
+    <t>Ativo Potencial</t>
+  </si>
+  <si>
+    <t>Percentual de Provisão</t>
+  </si>
+  <si>
+    <t>Provisão Constituída</t>
+  </si>
+  <si>
+    <t>Depósito Judicial Realizado?</t>
+  </si>
+  <si>
+    <t>CNPJ da Empresa Processada</t>
+  </si>
+  <si>
+    <t>Pagamento Realizado</t>
+  </si>
+  <si>
+    <t>Justificativa da Probabilidade</t>
+  </si>
+  <si>
     <t>Parâmetro</t>
   </si>
   <si>
@@ -331,6 +359,81 @@
     <t>Valor da causa − valor realizado, só dos encerrados com valor lançado.</t>
   </si>
   <si>
+    <t>Contingência</t>
+  </si>
+  <si>
+    <t>Passivo potencial total</t>
+  </si>
+  <si>
+    <t>Soma da coluna Passivo Potencial.</t>
+  </si>
+  <si>
+    <t>Passivo potencial dos processos ativos</t>
+  </si>
+  <si>
+    <t>Passivo Potencial dos processos com Ativo = Sim.</t>
+  </si>
+  <si>
+    <t>Passivo potencial atualizado (encerrados)</t>
+  </si>
+  <si>
+    <t>Soma da coluna Passivo Potencial Atualizado (correção e juros).</t>
+  </si>
+  <si>
+    <t>Provisão constituída total</t>
+  </si>
+  <si>
+    <t>Soma da coluna Provisão Constituída.</t>
+  </si>
+  <si>
+    <t>Ativo potencial total</t>
+  </si>
+  <si>
+    <t>Soma da coluna Ativo Potencial (créditos).</t>
+  </si>
+  <si>
+    <t>Passivo potencial (ativos): perda remota</t>
+  </si>
+  <si>
+    <t>Passivo Potencial dos processos ativos com Probabilidade = Remota.</t>
+  </si>
+  <si>
+    <t>Passivo potencial (ativos): perda possível</t>
+  </si>
+  <si>
+    <t>Passivo Potencial dos processos ativos com Probabilidade = Possível.</t>
+  </si>
+  <si>
+    <t>Passivo potencial (ativos): perda provável</t>
+  </si>
+  <si>
+    <t>Passivo Potencial dos processos ativos com Probabilidade = Provável.</t>
+  </si>
+  <si>
+    <t>Processos com depósito judicial</t>
+  </si>
+  <si>
+    <t>Coluna Depósito Judicial Realizado? = Sim.</t>
+  </si>
+  <si>
+    <t>Total de depósitos judiciais</t>
+  </si>
+  <si>
+    <t>Soma da coluna Depósitos Recursais (valor depositado).</t>
+  </si>
+  <si>
+    <t>Pagamentos realizados</t>
+  </si>
+  <si>
+    <t>Soma da coluna Pagamento Realizado.</t>
+  </si>
+  <si>
+    <t>Valor economizado</t>
+  </si>
+  <si>
+    <t>Soma da coluna Valor Economizado (passivo atualizado − pagamento).</t>
+  </si>
+  <si>
     <t>Processos por situação</t>
   </si>
   <si>
@@ -418,12 +521,24 @@
     <t>Remota</t>
   </si>
   <si>
+    <t>Passivo potencial dos ativos por probabilidade</t>
+  </si>
+  <si>
+    <t>Valor (R$)</t>
+  </si>
+  <si>
     <t>Resumo da carteira</t>
   </si>
   <si>
     <t>Ativos</t>
   </si>
   <si>
+    <t>Passivo potencial</t>
+  </si>
+  <si>
+    <t>Provisão constituída</t>
+  </si>
+  <si>
     <t>Data-base</t>
   </si>
   <si>
@@ -433,7 +548,25 @@
     <t>Valor estimado</t>
   </si>
   <si>
-    <t>Valor economizado</t>
+    <t>Grupo</t>
+  </si>
+  <si>
+    <t>Campo</t>
+  </si>
+  <si>
+    <t>Preenchidos</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Percentual</t>
+  </si>
+  <si>
+    <t>Origem</t>
+  </si>
+  <si>
+    <t>O que fazer</t>
   </si>
   <si>
     <t>Coluna de origem</t>
@@ -524,7 +657,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -537,6 +670,7 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -550,6 +684,7 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -686,12 +821,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Indicadores'!$A$36:$A$38</f>
+              <f>'Indicadores'!$A$50:$A$52</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Indicadores'!$B$36:$B$38</f>
+              <f>'Indicadores'!$B$50:$B$52</f>
             </numRef>
           </val>
         </ser>
@@ -777,12 +912,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Indicadores'!$A$41:$A$47</f>
+              <f>'Indicadores'!$A$55:$A$61</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Indicadores'!$B$41:$B$47</f>
+              <f>'Indicadores'!$B$55:$B$61</f>
             </numRef>
           </val>
         </ser>
@@ -868,12 +1003,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Indicadores'!$A$50:$A$61</f>
+              <f>'Indicadores'!$A$64:$A$75</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Indicadores'!$B$50:$B$61</f>
+              <f>'Indicadores'!$B$64:$B$75</f>
             </numRef>
           </val>
         </ser>
@@ -959,12 +1094,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Indicadores'!$A$64:$A$66</f>
+              <f>'Indicadores'!$A$78:$A$80</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Indicadores'!$B$64:$B$66</f>
+              <f>'Indicadores'!$B$78:$B$80</f>
             </numRef>
           </val>
         </ser>
@@ -1019,6 +1154,97 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Passivo potencial dos ativos por probabilidade (R$)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Indicadores'!$A$83:$A$85</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Indicadores'!$B$83:$B$85</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Valor (R$)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1233,7 +1459,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>0</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>37</row>
       <rowOff>0</rowOff>
@@ -1253,13 +1479,35 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProcessos" displayName="tblProcessos" ref="A1:AK2" headerRowCount="1">
-  <autoFilter ref="A1:AK2"/>
-  <tableColumns count="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProcessos" displayName="tblProcessos" ref="A1:AT2" headerRowCount="1">
+  <autoFilter ref="A1:AT2"/>
+  <tableColumns count="46">
     <tableColumn id="1" name="Número do Processo"/>
     <tableColumn id="2" name="Autor(es)"/>
     <tableColumn id="3" name="Réu(s)"/>
@@ -1301,6 +1549,15 @@
     <tableColumn id="35" name="Assunto"/>
     <tableColumn id="36" name="Valor do Acordo"/>
     <tableColumn id="37" name="Observações"/>
+    <tableColumn id="38" name="Passivo Potencial"/>
+    <tableColumn id="39" name="Passivo Potencial Atualizado"/>
+    <tableColumn id="40" name="Ativo Potencial"/>
+    <tableColumn id="41" name="Percentual de Provisão"/>
+    <tableColumn id="42" name="Provisão Constituída"/>
+    <tableColumn id="43" name="Depósito Judicial Realizado?"/>
+    <tableColumn id="44" name="CNPJ da Empresa Processada"/>
+    <tableColumn id="45" name="Pagamento Realizado"/>
+    <tableColumn id="46" name="Justificativa da Probabilidade"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -1323,7 +1580,23 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblNaoMigrados" displayName="tblNaoMigrados" ref="A1:C2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblFaltas" displayName="tblFaltas" ref="A1:G2" headerRowCount="1">
+  <autoFilter ref="A1:G2"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="Grupo"/>
+    <tableColumn id="2" name="Campo"/>
+    <tableColumn id="3" name="Preenchidos"/>
+    <tableColumn id="4" name="Total"/>
+    <tableColumn id="5" name="Percentual"/>
+    <tableColumn id="6" name="Origem"/>
+    <tableColumn id="7" name="O que fazer"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblNaoMigrados" displayName="tblNaoMigrados" ref="A1:C2" headerRowCount="1">
   <autoFilter ref="A1:C2"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Coluna de origem"/>
@@ -1623,7 +1896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK2"/>
+  <dimension ref="A1:AT2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1663,6 +1936,15 @@
     <col hidden="1" width="24" customWidth="1" min="35" max="35"/>
     <col hidden="1" width="16" customWidth="1" min="36" max="36"/>
     <col hidden="1" width="30" customWidth="1" min="37" max="37"/>
+    <col hidden="1" width="18" customWidth="1" min="38" max="38"/>
+    <col hidden="1" width="20" customWidth="1" min="39" max="39"/>
+    <col hidden="1" width="16" customWidth="1" min="40" max="40"/>
+    <col hidden="1" width="16" customWidth="1" min="41" max="41"/>
+    <col hidden="1" width="18" customWidth="1" min="42" max="42"/>
+    <col hidden="1" width="16" customWidth="1" min="43" max="43"/>
+    <col hidden="1" width="24" customWidth="1" min="44" max="44"/>
+    <col hidden="1" width="18" customWidth="1" min="45" max="45"/>
+    <col hidden="1" width="40" customWidth="1" min="46" max="46"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1776,6 +2058,33 @@
       </c>
       <c r="AK1" s="1" t="s">
         <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="2">
@@ -1822,6 +2131,15 @@
       <c r="AI2" s="2" t="n"/>
       <c r="AJ2" s="5" t="n"/>
       <c r="AK2" s="2" t="n"/>
+      <c r="AL2" s="5" t="n"/>
+      <c r="AM2" s="5" t="n"/>
+      <c r="AN2" s="5" t="n"/>
+      <c r="AO2" s="8" t="n"/>
+      <c r="AP2" s="5" t="n"/>
+      <c r="AQ2" s="2" t="n"/>
+      <c r="AR2" s="2" t="n"/>
+      <c r="AS2" s="5" t="n"/>
+      <c r="AT2" s="2" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="P2">
@@ -1835,12 +2153,12 @@
       <formula>$P2="Remota"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:AK2">
+  <conditionalFormatting sqref="A2:AT2">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>$N2="Não"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="8">
+  <dataValidations count="10">
     <dataValidation sqref="M2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Situação" error="Valor fora da lista padrão. Manter assim?" type="list" errorStyle="warning">
       <formula1>"Ativo,Encerrado,Suspenso"</formula1>
     </dataValidation>
@@ -1862,7 +2180,14 @@
     <dataValidation sqref="AB2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Reclamante terceirizado?" error="Valor fora da lista padrão. Manter assim?" type="list" errorStyle="warning">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
+    <dataValidation sqref="AQ2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Depósito Judicial Realizado?" error="Valor fora da lista padrão. Manter assim?" type="list" errorStyle="warning">
+      <formula1>"Sim,Não"</formula1>
+    </dataValidation>
     <dataValidation sqref="AA2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Percentual de êxito" error="Use uma fração entre 0 e 1 (0,85 = 85%)." type="decimal" errorStyle="warning" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation sqref="AO2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Percentual de Provisão" error="Use uma fração entre 0 e 1 (0,85 = 85%)." type="decimal" errorStyle="warning" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -1889,44 +2214,44 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>38</v>
+      <c r="A1" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" s="9" t="n"/>
+        <v>50</v>
+      </c>
+      <c r="B3" s="10" t="n"/>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1940,7 +2265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1949,590 +2274,774 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>48</v>
+      <c r="C1" s="9" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="s">
-        <v>49</v>
+      <c r="A2" s="11" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="11">
+        <v>59</v>
+      </c>
+      <c r="B3" s="12">
         <f>COUNTA(tblProcessos[Número do Processo])</f>
         <v/>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="11">
+        <v>61</v>
+      </c>
+      <c r="B4" s="12">
         <f>COUNTIFS(tblProcessos[Ativo],"Sim")</f>
         <v/>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="11">
+        <v>63</v>
+      </c>
+      <c r="B5" s="12">
         <f>COUNTIFS(tblProcessos[Ativo],"Não")</f>
         <v/>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="12">
+        <v>65</v>
+      </c>
+      <c r="B6" s="13">
         <f>IF(N('Parâmetros'!$B$2)&gt;0,B3/'Parâmetros'!$B$2*100,"")</f>
         <v/>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="11">
+        <v>67</v>
+      </c>
+      <c r="B7" s="12">
         <f>IF(N('Parâmetros'!$B$3)&gt;0,COUNTIFS(tblProcessos[Data do Ajuizamento],"&gt;"&amp;EDATE('Parâmetros'!$B$3,-12),tblProcessos[Data do Ajuizamento],"&lt;="&amp;'Parâmetros'!$B$3),"")</f>
         <v/>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="s">
-        <v>60</v>
+      <c r="A9" s="11" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>61</v>
-      </c>
-      <c r="B10" s="12">
+        <v>70</v>
+      </c>
+      <c r="B10" s="13">
         <f>IFERROR(AVERAGE(tblProcessos[[Taxa de resolução (em dias)]]),"")</f>
         <v/>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B11" s="12">
+        <v>72</v>
+      </c>
+      <c r="B11" s="13">
         <f>IFERROR(MEDIAN(tblProcessos[[Taxa de resolução (em dias)]]),"")</f>
         <v/>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B12" s="11">
+        <v>74</v>
+      </c>
+      <c r="B12" s="12">
         <f>COUNTIFS(tblProcessos[[Houve recurso da empresa?]],"Sim")</f>
         <v/>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>67</v>
-      </c>
-      <c r="B13" s="11">
+        <v>76</v>
+      </c>
+      <c r="B13" s="12">
         <f>B17+B18+B19+B20+B21</f>
         <v/>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>69</v>
-      </c>
-      <c r="B14" s="13">
+        <v>78</v>
+      </c>
+      <c r="B14" s="14">
         <f>IF(B13&gt;0,B12/B13,"")</f>
         <v/>
       </c>
       <c r="C14" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="s">
-        <v>71</v>
+      <c r="A16" s="11" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" s="11">
+        <v>81</v>
+      </c>
+      <c r="B17" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Improcedente")</f>
         <v/>
       </c>
       <c r="C17" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>74</v>
-      </c>
-      <c r="B18" s="11">
+        <v>83</v>
+      </c>
+      <c r="B18" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Arquivado / desistência")</f>
         <v/>
       </c>
       <c r="C18" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>76</v>
-      </c>
-      <c r="B19" s="11">
+        <v>85</v>
+      </c>
+      <c r="B19" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Acordo")</f>
         <v/>
       </c>
       <c r="C19" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>78</v>
-      </c>
-      <c r="B20" s="11">
+        <v>87</v>
+      </c>
+      <c r="B20" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Parcialmente procedente")</f>
         <v/>
       </c>
       <c r="C20" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>80</v>
-      </c>
-      <c r="B21" s="11">
+        <v>89</v>
+      </c>
+      <c r="B21" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Procedente")</f>
         <v/>
       </c>
       <c r="C21" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>82</v>
-      </c>
-      <c r="B22" s="13">
+        <v>91</v>
+      </c>
+      <c r="B22" s="14">
         <f>IF(B13&gt;0,(B17+B18)/B13,"")</f>
         <v/>
       </c>
       <c r="C22" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>84</v>
-      </c>
-      <c r="B23" s="13">
+        <v>93</v>
+      </c>
+      <c r="B23" s="14">
         <f>IF(B13&gt;0,B19/B13,"")</f>
         <v/>
       </c>
       <c r="C23" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="s">
-        <v>86</v>
+      <c r="A25" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>87</v>
-      </c>
-      <c r="B26" s="14">
+        <v>96</v>
+      </c>
+      <c r="B26" s="15">
         <f>SUM(tblProcessos[Valor da Causa])</f>
         <v/>
       </c>
       <c r="C26" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>89</v>
-      </c>
-      <c r="B27" s="14">
+        <v>98</v>
+      </c>
+      <c r="B27" s="15">
         <f>IF(N('Parâmetros'!$B$4)&gt;0,B26*'Parâmetros'!$B$4,B26)</f>
         <v/>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>91</v>
-      </c>
-      <c r="B28" s="14">
+        <v>100</v>
+      </c>
+      <c r="B28" s="15">
         <f>SUMIFS(tblProcessos[Valor da Causa],tblProcessos[Ativo],"Não")</f>
         <v/>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>93</v>
-      </c>
-      <c r="B29" s="11">
+        <v>102</v>
+      </c>
+      <c r="B29" s="12">
         <f>COUNTIFS(tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"&lt;&gt;")+COUNTIFS(tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"",tblProcessos[Valor da Execução],"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>95</v>
-      </c>
-      <c r="B30" s="11">
+        <v>104</v>
+      </c>
+      <c r="B30" s="12">
         <f>B5-B29</f>
         <v/>
       </c>
       <c r="C30" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>97</v>
-      </c>
-      <c r="B31" s="14">
+        <v>106</v>
+      </c>
+      <c r="B31" s="15">
         <f>SUMIFS(tblProcessos[Valor da Causa],tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"&lt;&gt;")+SUMIFS(tblProcessos[Valor da Causa],tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"",tblProcessos[Valor da Execução],"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C31" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>99</v>
-      </c>
-      <c r="B32" s="14">
+        <v>108</v>
+      </c>
+      <c r="B32" s="15">
         <f>SUMIFS(tblProcessos[Valor Arbitrado em Juízo],tblProcessos[Ativo],"Não")+SUMIFS(tblProcessos[Valor da Execução],tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"")</f>
         <v/>
       </c>
       <c r="C32" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>101</v>
-      </c>
-      <c r="B33" s="14">
+        <v>110</v>
+      </c>
+      <c r="B33" s="15">
         <f>B31-B32</f>
         <v/>
       </c>
       <c r="C33" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>104</v>
+      <c r="A35" s="11" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>13</v>
-      </c>
-      <c r="B36" s="11">
-        <f>COUNTIFS(tblProcessos[Situação],A36)</f>
-        <v/>
+        <v>113</v>
+      </c>
+      <c r="B36" s="15">
+        <f>SUM(tblProcessos[Passivo Potencial])</f>
+        <v/>
+      </c>
+      <c r="C36" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>105</v>
-      </c>
-      <c r="B37" s="11">
-        <f>COUNTIFS(tblProcessos[Situação],A37)</f>
-        <v/>
+        <v>115</v>
+      </c>
+      <c r="B37" s="15">
+        <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Ativo],"Sim")</f>
+        <v/>
+      </c>
+      <c r="C37" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>106</v>
-      </c>
-      <c r="B38" s="11">
-        <f>COUNTIFS(tblProcessos[Situação],A38)</f>
-        <v/>
+        <v>117</v>
+      </c>
+      <c r="B38" s="15">
+        <f>SUM(tblProcessos[Passivo Potencial Atualizado])</f>
+        <v/>
+      </c>
+      <c r="C38" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>119</v>
+      </c>
+      <c r="B39" s="15">
+        <f>SUM(tblProcessos[Provisão Constituída])</f>
+        <v/>
+      </c>
+      <c r="C39" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>104</v>
+      <c r="A40" t="s">
+        <v>121</v>
+      </c>
+      <c r="B40" s="15">
+        <f>SUM(tblProcessos[Ativo Potencial])</f>
+        <v/>
+      </c>
+      <c r="C40" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>108</v>
-      </c>
-      <c r="B41" s="11">
-        <f>COUNTIFS(tblProcessos[Resultado],A41)</f>
-        <v/>
+        <v>123</v>
+      </c>
+      <c r="B41" s="15">
+        <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],"Remota",tblProcessos[Ativo],"Sim")</f>
+        <v/>
+      </c>
+      <c r="C41" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>109</v>
-      </c>
-      <c r="B42" s="11">
-        <f>COUNTIFS(tblProcessos[Resultado],A42)</f>
-        <v/>
+        <v>125</v>
+      </c>
+      <c r="B42" s="15">
+        <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],"Possível",tblProcessos[Ativo],"Sim")</f>
+        <v/>
+      </c>
+      <c r="C42" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>110</v>
-      </c>
-      <c r="B43" s="11">
-        <f>COUNTIFS(tblProcessos[Resultado],A43)</f>
-        <v/>
+        <v>127</v>
+      </c>
+      <c r="B43" s="15">
+        <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],"Provável",tblProcessos[Ativo],"Sim")</f>
+        <v/>
+      </c>
+      <c r="C43" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>111</v>
-      </c>
-      <c r="B44" s="11">
-        <f>COUNTIFS(tblProcessos[Resultado],A44)</f>
-        <v/>
+        <v>129</v>
+      </c>
+      <c r="B44" s="12">
+        <f>COUNTIFS(tblProcessos[[Depósito Judicial Realizado?]],"Sim")</f>
+        <v/>
+      </c>
+      <c r="C44" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>112</v>
-      </c>
-      <c r="B45" s="11">
-        <f>COUNTIFS(tblProcessos[Resultado],A45)</f>
-        <v/>
+        <v>131</v>
+      </c>
+      <c r="B45" s="15">
+        <f>SUM(tblProcessos[Depósitos Recursais])</f>
+        <v/>
+      </c>
+      <c r="C45" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>113</v>
-      </c>
-      <c r="B46" s="11">
-        <f>COUNTIFS(tblProcessos[Resultado],A46)</f>
-        <v/>
+        <v>133</v>
+      </c>
+      <c r="B46" s="15">
+        <f>SUM(tblProcessos[Pagamento Realizado])</f>
+        <v/>
+      </c>
+      <c r="C46" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>114</v>
-      </c>
-      <c r="B47" s="11">
-        <f>COUNTIFS(tblProcessos[Resultado],A47)</f>
-        <v/>
+        <v>135</v>
+      </c>
+      <c r="B47" s="15">
+        <f>SUM(tblProcessos[Valor Economizado])</f>
+        <v/>
+      </c>
+      <c r="C47" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="B49" s="8" t="s">
-        <v>104</v>
+      <c r="A49" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>116</v>
-      </c>
-      <c r="B50" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A50)</f>
+        <v>13</v>
+      </c>
+      <c r="B50" s="12">
+        <f>COUNTIFS(tblProcessos[Situação],A50)</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>117</v>
-      </c>
-      <c r="B51" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A51)</f>
+        <v>139</v>
+      </c>
+      <c r="B51" s="12">
+        <f>COUNTIFS(tblProcessos[Situação],A51)</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>118</v>
-      </c>
-      <c r="B52" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A52)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="s">
-        <v>119</v>
-      </c>
-      <c r="B53" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A53)</f>
+        <v>140</v>
+      </c>
+      <c r="B52" s="12">
+        <f>COUNTIFS(tblProcessos[Situação],A52)</f>
         <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="s">
-        <v>120</v>
-      </c>
-      <c r="B54" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A54)</f>
-        <v/>
+      <c r="A54" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>121</v>
-      </c>
-      <c r="B55" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A55)</f>
+        <v>142</v>
+      </c>
+      <c r="B55" s="12">
+        <f>COUNTIFS(tblProcessos[Resultado],A55)</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>122</v>
-      </c>
-      <c r="B56" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A56)</f>
+        <v>143</v>
+      </c>
+      <c r="B56" s="12">
+        <f>COUNTIFS(tblProcessos[Resultado],A56)</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>123</v>
-      </c>
-      <c r="B57" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A57)</f>
+        <v>144</v>
+      </c>
+      <c r="B57" s="12">
+        <f>COUNTIFS(tblProcessos[Resultado],A57)</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>124</v>
-      </c>
-      <c r="B58" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A58)</f>
+        <v>145</v>
+      </c>
+      <c r="B58" s="12">
+        <f>COUNTIFS(tblProcessos[Resultado],A58)</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>125</v>
-      </c>
-      <c r="B59" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A59)</f>
+        <v>146</v>
+      </c>
+      <c r="B59" s="12">
+        <f>COUNTIFS(tblProcessos[Resultado],A59)</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>126</v>
-      </c>
-      <c r="B60" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A60)</f>
+        <v>147</v>
+      </c>
+      <c r="B60" s="12">
+        <f>COUNTIFS(tblProcessos[Resultado],A60)</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>127</v>
-      </c>
-      <c r="B61" s="11">
-        <f>COUNTIFS(tblProcessos[Área do Direito],A61)</f>
+        <v>148</v>
+      </c>
+      <c r="B61" s="12">
+        <f>COUNTIFS(tblProcessos[Resultado],A61)</f>
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="B63" s="8" t="s">
-        <v>104</v>
+      <c r="A63" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>129</v>
-      </c>
-      <c r="B64" s="11">
-        <f>COUNTIFS(tblProcessos[Probabilidade],A64)</f>
+        <v>150</v>
+      </c>
+      <c r="B64" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A64)</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>130</v>
-      </c>
-      <c r="B65" s="11">
-        <f>COUNTIFS(tblProcessos[Probabilidade],A65)</f>
+        <v>151</v>
+      </c>
+      <c r="B65" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A65)</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>131</v>
-      </c>
-      <c r="B66" s="11">
-        <f>COUNTIFS(tblProcessos[Probabilidade],A66)</f>
+        <v>152</v>
+      </c>
+      <c r="B66" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>153</v>
+      </c>
+      <c r="B67" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>154</v>
+      </c>
+      <c r="B68" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>155</v>
+      </c>
+      <c r="B69" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>156</v>
+      </c>
+      <c r="B70" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>157</v>
+      </c>
+      <c r="B71" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>158</v>
+      </c>
+      <c r="B72" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>159</v>
+      </c>
+      <c r="B73" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>160</v>
+      </c>
+      <c r="B74" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s">
+        <v>161</v>
+      </c>
+      <c r="B75" s="12">
+        <f>COUNTIFS(tblProcessos[Área do Direito],A75)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s">
+        <v>163</v>
+      </c>
+      <c r="B78" s="12">
+        <f>COUNTIFS(tblProcessos[Probabilidade],A78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>164</v>
+      </c>
+      <c r="B79" s="12">
+        <f>COUNTIFS(tblProcessos[Probabilidade],A79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>165</v>
+      </c>
+      <c r="B80" s="12">
+        <f>COUNTIFS(tblProcessos[Probabilidade],A80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B82" s="9" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s">
+        <v>163</v>
+      </c>
+      <c r="B83" s="15">
+        <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],A83,tblProcessos[Ativo],"Sim")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>164</v>
+      </c>
+      <c r="B84" s="15">
+        <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],A84,tblProcessos[Ativo],"Sim")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s">
+        <v>165</v>
+      </c>
+      <c r="B85" s="15">
+        <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],A85,tblProcessos[Ativo],"Sim")</f>
         <v/>
       </c>
     </row>
@@ -2547,7 +3056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2558,42 +3067,60 @@
     <col width="4" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="4" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="4" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="s">
-        <v>132</v>
+      <c r="A1" s="16" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>101</v>
+      <c r="A3" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17">
+      <c r="A4" s="18">
         <f>Indicadores!B3</f>
         <v/>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="18">
         <f>Indicadores!B4</f>
         <v/>
       </c>
-      <c r="E4" s="18">
+      <c r="E4" s="19">
         <f>Indicadores!B22</f>
         <v/>
       </c>
-      <c r="G4" s="19">
+      <c r="G4" s="20">
         <f>Indicadores!B33</f>
+        <v/>
+      </c>
+      <c r="I4" s="20">
+        <f>Indicadores!B36</f>
+        <v/>
+      </c>
+      <c r="K4" s="20">
+        <f>Indicadores!B39</f>
         <v/>
       </c>
     </row>
@@ -2622,26 +3149,26 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="s">
-        <v>134</v>
-      </c>
-      <c r="B1" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="C1" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="D1" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="20" t="s">
+      <c r="A1" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>173</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="G1" s="21" t="s">
         <v>135</v>
-      </c>
-      <c r="F1" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="G1" s="20" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="2">
@@ -2667,6 +3194,60 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" s="12" t="n"/>
+      <c r="D2" s="12" t="n"/>
+      <c r="E2" s="22" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2676,14 +3257,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="s">
-        <v>138</v>
-      </c>
-      <c r="B1" s="20" t="s">
-        <v>139</v>
-      </c>
-      <c r="C1" s="20" t="s">
-        <v>38</v>
+      <c r="A1" s="21" t="s">
+        <v>182</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Campo grau_tramitacao: sinal do relatório para ler o 2º grau/TST
Vocabulário e campo da ficha (grupo situação), leitura da coluna (sem colidir
com grau de risco/probabilidade), coluna "Grau de Tramitação" no modelo B
(extra no fim, ativada quando há valor), sinal da ficha até o pje_trt
(proc["sinal_grau"] em trt.indicio_de_recurso) e atualização automática pelo
resultado da coleta (maior grau lido; humano não é sobrescrito; nunca rebaixa).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/modelos/xlsx_b/modelo_padrao.xlsx
+++ b/src/modelos/xlsx_b/modelo_padrao.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="185">
   <si>
     <t>Número do Processo</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>Justificativa da Probabilidade</t>
+  </si>
+  <si>
+    <t>Grau de Tramitação</t>
   </si>
   <si>
     <t>Parâmetro</t>
@@ -1505,9 +1508,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProcessos" displayName="tblProcessos" ref="A1:AT2" headerRowCount="1">
-  <autoFilter ref="A1:AT2"/>
-  <tableColumns count="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblProcessos" displayName="tblProcessos" ref="A1:AU2" headerRowCount="1">
+  <autoFilter ref="A1:AU2"/>
+  <tableColumns count="47">
     <tableColumn id="1" name="Número do Processo"/>
     <tableColumn id="2" name="Autor(es)"/>
     <tableColumn id="3" name="Réu(s)"/>
@@ -1558,6 +1561,7 @@
     <tableColumn id="44" name="CNPJ da Empresa Processada"/>
     <tableColumn id="45" name="Pagamento Realizado"/>
     <tableColumn id="46" name="Justificativa da Probabilidade"/>
+    <tableColumn id="47" name="Grau de Tramitação"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -1896,7 +1900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT2"/>
+  <dimension ref="A1:AU2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1945,6 +1949,7 @@
     <col hidden="1" width="24" customWidth="1" min="44" max="44"/>
     <col hidden="1" width="18" customWidth="1" min="45" max="45"/>
     <col hidden="1" width="40" customWidth="1" min="46" max="46"/>
+    <col hidden="1" width="16" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2085,6 +2090,9 @@
       </c>
       <c r="AT1" s="1" t="s">
         <v>45</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="2">
@@ -2140,6 +2148,7 @@
       <c r="AR2" s="2" t="n"/>
       <c r="AS2" s="5" t="n"/>
       <c r="AT2" s="2" t="n"/>
+      <c r="AU2" s="2" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="P2">
@@ -2153,12 +2162,12 @@
       <formula>$P2="Remota"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:AT2">
+  <conditionalFormatting sqref="A2:AU2">
     <cfRule type="expression" priority="4" dxfId="3">
       <formula>$N2="Não"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="10">
+  <dataValidations count="11">
     <dataValidation sqref="M2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Situação" error="Valor fora da lista padrão. Manter assim?" type="list" errorStyle="warning">
       <formula1>"Ativo,Encerrado,Suspenso"</formula1>
     </dataValidation>
@@ -2182,6 +2191,9 @@
     </dataValidation>
     <dataValidation sqref="AQ2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Depósito Judicial Realizado?" error="Valor fora da lista padrão. Manter assim?" type="list" errorStyle="warning">
       <formula1>"Sim,Não"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AU2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Grau de Tramitação" error="Valor fora da lista padrão. Manter assim?" type="list" errorStyle="warning">
+      <formula1>"1º grau,2º grau,TST"</formula1>
     </dataValidation>
     <dataValidation sqref="AA2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Percentual de êxito" error="Use uma fração entre 0 e 1 (0,85 = 85%)." type="decimal" errorStyle="warning" operator="between">
       <formula1>0</formula1>
@@ -2215,43 +2227,43 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B3" s="10" t="n"/>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2275,490 +2287,490 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B3" s="12">
         <f>COUNTA(tblProcessos[Número do Processo])</f>
         <v/>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B4" s="12">
         <f>COUNTIFS(tblProcessos[Ativo],"Sim")</f>
         <v/>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B5" s="12">
         <f>COUNTIFS(tblProcessos[Ativo],"Não")</f>
         <v/>
       </c>
       <c r="C5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B6" s="13">
         <f>IF(N('Parâmetros'!$B$2)&gt;0,B3/'Parâmetros'!$B$2*100,"")</f>
         <v/>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B7" s="12">
         <f>IF(N('Parâmetros'!$B$3)&gt;0,COUNTIFS(tblProcessos[Data do Ajuizamento],"&gt;"&amp;EDATE('Parâmetros'!$B$3,-12),tblProcessos[Data do Ajuizamento],"&lt;="&amp;'Parâmetros'!$B$3),"")</f>
         <v/>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B10" s="13">
         <f>IFERROR(AVERAGE(tblProcessos[[Taxa de resolução (em dias)]]),"")</f>
         <v/>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B11" s="13">
         <f>IFERROR(MEDIAN(tblProcessos[[Taxa de resolução (em dias)]]),"")</f>
         <v/>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12" s="12">
         <f>COUNTIFS(tblProcessos[[Houve recurso da empresa?]],"Sim")</f>
         <v/>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B13" s="12">
         <f>B17+B18+B19+B20+B21</f>
         <v/>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B14" s="14">
         <f>IF(B13&gt;0,B12/B13,"")</f>
         <v/>
       </c>
       <c r="C14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B17" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Improcedente")</f>
         <v/>
       </c>
       <c r="C17" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B18" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Arquivado / desistência")</f>
         <v/>
       </c>
       <c r="C18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B19" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Acordo")</f>
         <v/>
       </c>
       <c r="C19" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B20" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Parcialmente procedente")</f>
         <v/>
       </c>
       <c r="C20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B21" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],"Procedente")</f>
         <v/>
       </c>
       <c r="C21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B22" s="14">
         <f>IF(B13&gt;0,(B17+B18)/B13,"")</f>
         <v/>
       </c>
       <c r="C22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B23" s="14">
         <f>IF(B13&gt;0,B19/B13,"")</f>
         <v/>
       </c>
       <c r="C23" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B26" s="15">
         <f>SUM(tblProcessos[Valor da Causa])</f>
         <v/>
       </c>
       <c r="C26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B27" s="15">
         <f>IF(N('Parâmetros'!$B$4)&gt;0,B26*'Parâmetros'!$B$4,B26)</f>
         <v/>
       </c>
       <c r="C27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B28" s="15">
         <f>SUMIFS(tblProcessos[Valor da Causa],tblProcessos[Ativo],"Não")</f>
         <v/>
       </c>
       <c r="C28" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B29" s="12">
         <f>COUNTIFS(tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"&lt;&gt;")+COUNTIFS(tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"",tblProcessos[Valor da Execução],"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C29" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B30" s="12">
         <f>B5-B29</f>
         <v/>
       </c>
       <c r="C30" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B31" s="15">
         <f>SUMIFS(tblProcessos[Valor da Causa],tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"&lt;&gt;")+SUMIFS(tblProcessos[Valor da Causa],tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"",tblProcessos[Valor da Execução],"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C31" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B32" s="15">
         <f>SUMIFS(tblProcessos[Valor Arbitrado em Juízo],tblProcessos[Ativo],"Não")+SUMIFS(tblProcessos[Valor da Execução],tblProcessos[Ativo],"Não",tblProcessos[Valor Arbitrado em Juízo],"")</f>
         <v/>
       </c>
       <c r="C32" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B33" s="15">
         <f>B31-B32</f>
         <v/>
       </c>
       <c r="C33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B36" s="15">
         <f>SUM(tblProcessos[Passivo Potencial])</f>
         <v/>
       </c>
       <c r="C36" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B37" s="15">
         <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Ativo],"Sim")</f>
         <v/>
       </c>
       <c r="C37" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B38" s="15">
         <f>SUM(tblProcessos[Passivo Potencial Atualizado])</f>
         <v/>
       </c>
       <c r="C38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B39" s="15">
         <f>SUM(tblProcessos[Provisão Constituída])</f>
         <v/>
       </c>
       <c r="C39" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B40" s="15">
         <f>SUM(tblProcessos[Ativo Potencial])</f>
         <v/>
       </c>
       <c r="C40" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B41" s="15">
         <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],"Remota",tblProcessos[Ativo],"Sim")</f>
         <v/>
       </c>
       <c r="C41" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B42" s="15">
         <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],"Possível",tblProcessos[Ativo],"Sim")</f>
         <v/>
       </c>
       <c r="C42" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B43" s="15">
         <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],"Provável",tblProcessos[Ativo],"Sim")</f>
         <v/>
       </c>
       <c r="C43" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B44" s="12">
         <f>COUNTIFS(tblProcessos[[Depósito Judicial Realizado?]],"Sim")</f>
         <v/>
       </c>
       <c r="C44" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B45" s="15">
         <f>SUM(tblProcessos[Depósitos Recursais])</f>
         <v/>
       </c>
       <c r="C45" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B46" s="15">
         <f>SUM(tblProcessos[Pagamento Realizado])</f>
         <v/>
       </c>
       <c r="C46" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B47" s="15">
         <f>SUM(tblProcessos[Valor Economizado])</f>
         <v/>
       </c>
       <c r="C47" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="50">
@@ -2772,7 +2784,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B51" s="12">
         <f>COUNTIFS(tblProcessos[Situação],A51)</f>
@@ -2781,7 +2793,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B52" s="12">
         <f>COUNTIFS(tblProcessos[Situação],A52)</f>
@@ -2790,15 +2802,15 @@
     </row>
     <row r="54">
       <c r="A54" s="11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B55" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],A55)</f>
@@ -2807,7 +2819,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B56" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],A56)</f>
@@ -2816,7 +2828,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B57" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],A57)</f>
@@ -2825,7 +2837,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B58" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],A58)</f>
@@ -2834,7 +2846,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B59" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],A59)</f>
@@ -2843,7 +2855,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B60" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],A60)</f>
@@ -2852,7 +2864,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B61" s="12">
         <f>COUNTIFS(tblProcessos[Resultado],A61)</f>
@@ -2861,15 +2873,15 @@
     </row>
     <row r="63">
       <c r="A63" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B64" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A64)</f>
@@ -2878,7 +2890,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B65" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A65)</f>
@@ -2887,7 +2899,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B66" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A66)</f>
@@ -2896,7 +2908,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B67" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A67)</f>
@@ -2905,7 +2917,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B68" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A68)</f>
@@ -2914,7 +2926,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B69" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A69)</f>
@@ -2923,7 +2935,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B70" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A70)</f>
@@ -2932,7 +2944,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B71" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A71)</f>
@@ -2941,7 +2953,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B72" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A72)</f>
@@ -2950,7 +2962,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B73" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A73)</f>
@@ -2959,7 +2971,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B74" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A74)</f>
@@ -2968,7 +2980,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B75" s="12">
         <f>COUNTIFS(tblProcessos[Área do Direito],A75)</f>
@@ -2977,15 +2989,15 @@
     </row>
     <row r="77">
       <c r="A77" s="11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B77" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B78" s="12">
         <f>COUNTIFS(tblProcessos[Probabilidade],A78)</f>
@@ -2994,7 +3006,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B79" s="12">
         <f>COUNTIFS(tblProcessos[Probabilidade],A79)</f>
@@ -3003,7 +3015,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B80" s="12">
         <f>COUNTIFS(tblProcessos[Probabilidade],A80)</f>
@@ -3012,15 +3024,15 @@
     </row>
     <row r="82">
       <c r="A82" s="11" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B83" s="15">
         <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],A83,tblProcessos[Ativo],"Sim")</f>
@@ -3029,7 +3041,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B84" s="15">
         <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],A84,tblProcessos[Ativo],"Sim")</f>
@@ -3038,7 +3050,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B85" s="15">
         <f>SUMIFS(tblProcessos[Passivo Potencial],tblProcessos[Probabilidade],A85,tblProcessos[Ativo],"Sim")</f>
@@ -3075,27 +3087,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="16" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="17" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4">
@@ -3150,25 +3162,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2">
@@ -3208,25 +3220,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E1" s="21" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2">
@@ -3258,13 +3270,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="21" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>